<commit_message>
Add cell comment tooltips to all 28 template header columns
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/MarginCOS_Sample_Template_FMCG.xlsx
+++ b/public/downloads/MarginCOS_Sample_Template_FMCG.xlsx
@@ -221,6 +221,156 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>MarginCOS</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t>Your internal product code. Must be unique.</t>
+      </text>
+    </comment>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>Full product name as it appears on-pack or in your ERP.</t>
+      </text>
+    </comment>
+    <comment ref="C2" authorId="0" shapeId="0">
+      <text>
+        <t>Product category from your vertical's taxonomy.</t>
+      </text>
+    </comment>
+    <comment ref="D2" authorId="0" shapeId="0">
+      <text>
+        <t>Recommended Retail Price in Naira per unit.</t>
+      </text>
+    </comment>
+    <comment ref="E2" authorId="0" shapeId="0">
+      <text>
+        <t>Include in analysis. Y = active, N = excluded.</t>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="0" shapeId="0">
+      <text>
+        <t>Price positioning: Mass Market, Mid-Range, or Premium.</t>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="0" shapeId="0">
+      <text>
+        <t>Division or brand cluster.</t>
+      </text>
+    </comment>
+    <comment ref="H2" authorId="0" shapeId="0">
+      <text>
+        <t>Primary geographic region.</t>
+      </text>
+    </comment>
+    <comment ref="I2" authorId="0" shapeId="0">
+      <text>
+        <t>Nearest competitor's shelf price.</t>
+      </text>
+    </comment>
+    <comment ref="J2" authorId="0" shapeId="0">
+      <text>
+        <t>Minimum acceptable gross margin %.</t>
+      </text>
+    </comment>
+    <comment ref="K2" authorId="0" shapeId="0">
+      <text>
+        <t>Demand sensitivity to price change.</t>
+      </text>
+    </comment>
+    <comment ref="L2" authorId="0" shapeId="0">
+      <text>
+        <t>Proposed price increase/decrease %.</t>
+      </text>
+    </comment>
+    <comment ref="M2" authorId="0" shapeId="0">
+      <text>
+        <t>Willingness-to-pay premium %.</t>
+      </text>
+    </comment>
+    <comment ref="N2" authorId="0" shapeId="0">
+      <text>
+        <t>Cost of Goods Sold per unit.</t>
+      </text>
+    </comment>
+    <comment ref="O2" authorId="0" shapeId="0">
+      <text>
+        <t>COGS per unit in the previous period.</t>
+      </text>
+    </comment>
+    <comment ref="P2" authorId="0" shapeId="0">
+      <text>
+        <t>Annual input cost inflation rate.</t>
+      </text>
+    </comment>
+    <comment ref="Q2" authorId="0" shapeId="0">
+      <text>
+        <t>% of cost increase passed on to trade.</t>
+      </text>
+    </comment>
+    <comment ref="R2" authorId="0" shapeId="0">
+      <text>
+        <t>% of COGS linked to foreign currency.</t>
+      </text>
+    </comment>
+    <comment ref="S2" authorId="0" shapeId="0">
+      <text>
+        <t>Primary route-to-market.</t>
+      </text>
+    </comment>
+    <comment ref="T2" authorId="0" shapeId="0">
+      <text>
+        <t>% of volume through primary channel.</t>
+      </text>
+    </comment>
+    <comment ref="U2" authorId="0" shapeId="0">
+      <text>
+        <t>Primary distributor name.</t>
+      </text>
+    </comment>
+    <comment ref="V2" authorId="0" shapeId="0">
+      <text>
+        <t>Distributor margin %.</t>
+      </text>
+    </comment>
+    <comment ref="W2" authorId="0" shapeId="0">
+      <text>
+        <t>Retrospective rebate %.</t>
+      </text>
+    </comment>
+    <comment ref="X2" authorId="0" shapeId="0">
+      <text>
+        <t>Delivery cost per unit.</t>
+      </text>
+    </comment>
+    <comment ref="Y2" authorId="0" shapeId="0">
+      <text>
+        <t>Payment terms in days.</t>
+      </text>
+    </comment>
+    <comment ref="Z2" authorId="0" shapeId="0">
+      <text>
+        <t>Units sold in the period.</t>
+      </text>
+    </comment>
+    <comment ref="AA2" authorId="0" shapeId="0">
+      <text>
+        <t>Promotional discount %.</t>
+      </text>
+    </comment>
+    <comment ref="AB2" authorId="0" shapeId="0">
+      <text>
+        <t>Expected volume uplift %.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2156,5 +2306,6 @@
   </sheetData>
   <autoFilter ref="A2:AB7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>